<commit_message>
Add voltage drop calculation for transmitter power supply cables
Calculates voltage at transmitter terminals accounting for:
- Cable 9 (250m) carrying combined current of both transmitters
- Cable 3/4 (15m) individual feeds
- Temperature derating (20-65°C, India climate)
- 4 load scenarios (60-200 mA per transmitter)

Worst case (150mA, 65°C): 21.88V at transmitter (within 18-30V spec).
Added as Sheet 6 in Excel file + standalone calculation script.

https://claude.ai/code/session_011Zercr8tn7pWHAp5jBVCSm
</commit_message>
<xml_diff>
--- a/K1_Cable_Journal.xlsx
+++ b/K1_Cable_Journal.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клеммные карты" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка материалов" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Замечания" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Падение напряжения" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +66,33 @@
       <color rgb="00CC0000"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -145,6 +171,30 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -170,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -243,6 +293,61 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3318,4 +3423,982 @@
   <pageMargins left="0.5" right="0.5" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF6600"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>РАСЧЁТ ПАДЕНИЯ НАПРЯЖЕНИЯ В КАБЕЛЯХ ПИТАНИЯ / VOLTAGE DROP CALCULATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DEEPAK K1 — GP Plant  |  421457.103E1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>СХЕМА ЦЕПИ ПИТАНИЯ ТРАНСМИТТЕРОВ</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="24" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="24" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>SCADA Ekor Box (24VDC) ──[ Cable 9: 250м, 1.5мм² ]──&gt; Connection Box ──[ Cable 3: 15м ]──&gt; Трансмиттер №1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                                          └──[ Cable 4: 15м ]──&gt; Трансмиттер №2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>ВАЖНО: Cable 9 несёт суммарный ток ОБОИХ трансмиттеров!</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="24" t="n"/>
+      <c r="F7" s="24" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>ИСХОДНЫЕ ДАННЫЕ</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Напряжение источника (SCADA Ekor Box)</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>24.0 В</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Удельное сопротивление меди при 20°C (ρ₂₀)</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>0.0175 Ом·мм²/м</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="24" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Температурный коэффициент меди (α)</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>0.00393 1/°C</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="24" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Cable 9: длина / сечение</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>250 м / 1.5 мм²</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="24" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Cable 3: длина / сечение</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>15 м / 1.5 мм²</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="24" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Cable 4: длина / сечение</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>15 м / 1.5 мм²</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="24" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Допустимый диапазон питания трансмиттера</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>18...30 В</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Рекомендуемый минимум (с запасом на пульсации)</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>20 В</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="24" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>ПОТРЕБЛЕНИЕ ТОКА ТРАНСМИТТЕРА (РАЗБИВКА)</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="24" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>Электроника трансмиттера (MCU, АЦП, ЦАП)</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>~80 мА</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="24" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>RS-485 приёмопередатчик</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>~15 мА</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
+      <c r="F21" s="24" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>Выход 4-20 мА QS1 (Потенциал/ORP)</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>4...20 мА</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
+      <c r="F22" s="24" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>Выход 4-20 мА QS2 (pH/Концентрация)</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>4...20 мА</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
+      <c r="F23" s="24" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="inlineStr">
+        <is>
+          <t>Запас на пульсации и потери в стабилизаторе</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>~15 мА</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="24" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>СОПРОТИВЛЕНИЕ КАБЕЛЕЙ (одна жила, Ом)</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="F26" s="24" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Кабель</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>R@20°C</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>R@35°C</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>R@50°C</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>R@65°C</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>R петли@50°C</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Cable 9 (250м, 1.5мм²)</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>2.917</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>3.089</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>3.261</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>3.432</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>6.521</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Cable 3 (15м, 1.5мм²)</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>0.391</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Cable 4 (15м, 1.5мм²)</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>0.391</v>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="33" t="inlineStr">
+        <is>
+          <t>СВОДНАЯ ТАБЛИЦА: НАПРЯЖЕНИЕ НА КЛЕММАХ ТРАНСМИТТЕРА (В)</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Режим работы</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>I транс., мА</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>20°C</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>35°C</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>50°C</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>65°C</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Минимальный (холостой ход, выходы 4мА)</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="n">
+        <v>60</v>
+      </c>
+      <c r="C34" s="34" t="n">
+        <v>23.28</v>
+      </c>
+      <c r="D34" s="34" t="n">
+        <v>23.24</v>
+      </c>
+      <c r="E34" s="34" t="n">
+        <v>23.19</v>
+      </c>
+      <c r="F34" s="34" t="n">
+        <v>23.15</v>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Номинальный (выходы ~12мА)</t>
+        </is>
+      </c>
+      <c r="B35" s="31" t="n">
+        <v>120</v>
+      </c>
+      <c r="C35" s="34" t="n">
+        <v>22.56</v>
+      </c>
+      <c r="D35" s="34" t="n">
+        <v>22.47</v>
+      </c>
+      <c r="E35" s="34" t="n">
+        <v>22.39</v>
+      </c>
+      <c r="F35" s="34" t="n">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Максимальный (выходы 20мА, полная нагрузка)</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="n">
+        <v>150</v>
+      </c>
+      <c r="C36" s="34" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D36" s="34" t="n">
+        <v>22.09</v>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="F36" s="34" t="n">
+        <v>21.88</v>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>Аварийный (пусковой бросок)</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="n">
+        <v>200</v>
+      </c>
+      <c r="C37" s="34" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="E37" s="34" t="n">
+        <v>21.31</v>
+      </c>
+      <c r="F37" s="34" t="n">
+        <v>21.17</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>Цветовая шкала:</t>
+        </is>
+      </c>
+      <c r="C38" s="36" t="inlineStr">
+        <is>
+          <t>&gt; 20 В</t>
+        </is>
+      </c>
+      <c r="D38" s="37" t="inlineStr">
+        <is>
+          <t>&lt; 20 В</t>
+        </is>
+      </c>
+      <c r="E38" s="38" t="inlineStr">
+        <is>
+          <t>&lt; 18 В</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="39" t="inlineStr">
+        <is>
+          <t>ДЕТАЛЬНЫЙ РАСЧЁТ — НАИХУДШИЙ СЛУЧАЙ (150 мА, 65°C)</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="40" t="inlineStr">
+        <is>
+          <t>Ток одного трансмиттера</t>
+        </is>
+      </c>
+      <c r="B41" s="41" t="inlineStr">
+        <is>
+          <t>150 мА</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="40" t="inlineStr">
+        <is>
+          <t>Суммарный ток в Cable 9 (оба трансмиттера)</t>
+        </is>
+      </c>
+      <c r="B42" s="41" t="inlineStr">
+        <is>
+          <t>300 мА</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="F42" s="24" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="40" t="inlineStr">
+        <is>
+          <t>R(Cable 9) при 65°C — одна жила</t>
+        </is>
+      </c>
+      <c r="B43" s="41" t="inlineStr">
+        <is>
+          <t>3.432 Ом</t>
+        </is>
+      </c>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="24" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>R(Cable 9) при 65°C — петля (туда+обратно)</t>
+        </is>
+      </c>
+      <c r="B44" s="41" t="inlineStr">
+        <is>
+          <t>6.865 Ом</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="n"/>
+      <c r="D44" s="24" t="n"/>
+      <c r="E44" s="24" t="n"/>
+      <c r="F44" s="24" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="40" t="inlineStr">
+        <is>
+          <t>R(Cable 3/4) при 65°C — петля</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="inlineStr">
+        <is>
+          <t>0.412 Ом</t>
+        </is>
+      </c>
+      <c r="C45" s="24" t="n"/>
+      <c r="D45" s="24" t="n"/>
+      <c r="E45" s="24" t="n"/>
+      <c r="F45" s="24" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="42" t="inlineStr"/>
+      <c r="B46" s="43" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="40" t="inlineStr">
+        <is>
+          <t>ΔU на Cable 9 (250 м)</t>
+        </is>
+      </c>
+      <c r="B47" s="41" t="inlineStr">
+        <is>
+          <t>2.06 В</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="n"/>
+      <c r="D47" s="24" t="n"/>
+      <c r="E47" s="24" t="n"/>
+      <c r="F47" s="24" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="40" t="inlineStr">
+        <is>
+          <t>ΔU на Cable 3/4 (15 м)</t>
+        </is>
+      </c>
+      <c r="B48" s="41" t="inlineStr">
+        <is>
+          <t>0.06 В</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="n"/>
+      <c r="D48" s="24" t="n"/>
+      <c r="E48" s="24" t="n"/>
+      <c r="F48" s="24" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="44" t="inlineStr">
+        <is>
+          <t>ИТОГО падение напряжения</t>
+        </is>
+      </c>
+      <c r="B49" s="45" t="inlineStr">
+        <is>
+          <t>2.12 В  (8.8%)</t>
+        </is>
+      </c>
+      <c r="C49" s="24" t="n"/>
+      <c r="D49" s="24" t="n"/>
+      <c r="E49" s="24" t="n"/>
+      <c r="F49" s="24" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="42" t="inlineStr"/>
+      <c r="B50" s="43" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="40" t="inlineStr">
+        <is>
+          <t>V на Connection Box</t>
+        </is>
+      </c>
+      <c r="B51" s="41" t="inlineStr">
+        <is>
+          <t>21.94 В</t>
+        </is>
+      </c>
+      <c r="C51" s="24" t="n"/>
+      <c r="D51" s="24" t="n"/>
+      <c r="E51" s="24" t="n"/>
+      <c r="F51" s="24" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="44" t="inlineStr">
+        <is>
+          <t>V НА ТРАНСМИТТЕРЕ</t>
+        </is>
+      </c>
+      <c r="B52" s="45" t="inlineStr">
+        <is>
+          <t>21.88 В</t>
+        </is>
+      </c>
+      <c r="C52" s="24" t="n"/>
+      <c r="D52" s="24" t="n"/>
+      <c r="E52" s="24" t="n"/>
+      <c r="F52" s="24" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="42" t="inlineStr"/>
+      <c r="B53" s="43" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="40" t="inlineStr">
+        <is>
+          <t>Мощность потерь в Cable 9</t>
+        </is>
+      </c>
+      <c r="B54" s="41" t="inlineStr">
+        <is>
+          <t>0.62 Вт</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="n"/>
+      <c r="D54" s="24" t="n"/>
+      <c r="E54" s="24" t="n"/>
+      <c r="F54" s="24" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="40" t="inlineStr">
+        <is>
+          <t>Мощность потерь в Cable 3/4</t>
+        </is>
+      </c>
+      <c r="B55" s="41" t="inlineStr">
+        <is>
+          <t>0.009 Вт</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="n"/>
+      <c r="D55" s="24" t="n"/>
+      <c r="E55" s="24" t="n"/>
+      <c r="F55" s="24" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="40" t="inlineStr">
+        <is>
+          <t>Суммарные тепловые потери</t>
+        </is>
+      </c>
+      <c r="B56" s="41" t="inlineStr">
+        <is>
+          <t>0.63 Вт</t>
+        </is>
+      </c>
+      <c r="C56" s="24" t="n"/>
+      <c r="D56" s="24" t="n"/>
+      <c r="E56" s="24" t="n"/>
+      <c r="F56" s="24" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="46" t="inlineStr">
+        <is>
+          <t>РЕКОМЕНДАЦИИ / RECOMMENDATIONS</t>
+        </is>
+      </c>
+      <c r="B58" s="24" t="n"/>
+      <c r="C58" s="24" t="n"/>
+      <c r="D58" s="24" t="n"/>
+      <c r="E58" s="24" t="n"/>
+      <c r="F58" s="24" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Рекомендация</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>V, В</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Падение, В</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>1. Увеличить сечение Cable 9 до 2.5 мм²</t>
+        </is>
+      </c>
+      <c r="B60" s="32" t="inlineStr">
+        <is>
+          <t>V на трансмиттере (65°C, 150мА)</t>
+        </is>
+      </c>
+      <c r="C60" s="34" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D60" s="14" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E60" s="47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>2. Повысить напряжение источника до 27 В</t>
+        </is>
+      </c>
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>V на трансмиттере (65°C, 150мА)</t>
+        </is>
+      </c>
+      <c r="C61" s="34" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="D61" s="14" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="E61" s="47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
+          <t>3. Сократить Cable 9 до 100 м (перенести SCADA box)</t>
+        </is>
+      </c>
+      <c r="B62" s="32" t="inlineStr">
+        <is>
+          <t>V на трансмиттере (65°C, 150мА)</t>
+        </is>
+      </c>
+      <c r="C62" s="34" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="D62" s="14" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="E62" s="47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>4. Отдельный БП 24VDC у Connection Box</t>
+        </is>
+      </c>
+      <c r="B63" s="32" t="inlineStr">
+        <is>
+          <t>V на трансмиттере (без Cable 9)</t>
+        </is>
+      </c>
+      <c r="C63" s="34" t="n">
+        <v>23.94</v>
+      </c>
+      <c r="D63" s="14" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E63" s="47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="41">
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix voltage drop calc: use actual 350mA (8W) from K1 documentation
Previous calculation used estimated 60-200mA. K1 technical description
specifies "Power consumption of the transmitter: 8 W (0.35A)".

With 350mA per transmitter (700mA total in Cable 9, 250m):
- At 20°C: 19.79V (below recommended 20V minimum!)
- At 50°C: 19.30V
- At 65°C: 19.05V (only 1.05V above absolute minimum 18V)

This reveals a real design concern with 1.5mm² cable at 250m.

https://claude.ai/code/session_011Zercr8tn7pWHAp5jBVCSm
</commit_message>
<xml_diff>
--- a/K1_Cable_Journal.xlsx
+++ b/K1_Cable_Journal.xlsx
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -310,6 +310,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3432,7 +3435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3638,7 +3641,7 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>ПОТРЕБЛЕНИЕ ТОКА ТРАНСМИТТЕРА (РАЗБИВКА)</t>
+          <t>ПОТРЕБЛЕНИЕ ТОКА ТРАНСМИТТЕРА (из документации K1)</t>
         </is>
       </c>
       <c r="B19" s="24" t="n"/>
@@ -3650,12 +3653,12 @@
     <row r="20">
       <c r="A20" s="32" t="inlineStr">
         <is>
-          <t>Электроника трансмиттера (MCU, АЦП, ЦАП)</t>
+          <t>Паспортное: "Power consumption of the transmitter: 8 W (0.35A)"</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>~80 мА</t>
+          <t>350 мА (8 Вт / 24 В)</t>
         </is>
       </c>
       <c r="C20" s="24" t="n"/>
@@ -3666,14 +3669,10 @@
     <row r="21">
       <c r="A21" s="32" t="inlineStr">
         <is>
-          <t>RS-485 приёмопередатчик</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>~15 мА</t>
-        </is>
-      </c>
+          <t>I = P / U = 8 Вт / 24 В = 0.333 А (округлено до 0.35 А)</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr"/>
       <c r="C21" s="24" t="n"/>
       <c r="D21" s="24" t="n"/>
       <c r="E21" s="24" t="n"/>
@@ -3682,12 +3681,12 @@
     <row r="22">
       <c r="A22" s="32" t="inlineStr">
         <is>
-          <t>Выход 4-20 мА QS1 (Потенциал/ORP)</t>
+          <t>Суммарный ток в Cable 9 (два трансмиттера)</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>4...20 мА</t>
+          <t>700 мА</t>
         </is>
       </c>
       <c r="C22" s="24" t="n"/>
@@ -3695,323 +3694,323 @@
       <c r="E22" s="24" t="n"/>
       <c r="F22" s="24" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="32" t="inlineStr">
-        <is>
-          <t>Выход 4-20 мА QS2 (pH/Концентрация)</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>4...20 мА</t>
-        </is>
-      </c>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
-    </row>
     <row r="24">
-      <c r="A24" s="32" t="inlineStr">
-        <is>
-          <t>Запас на пульсации и потери в стабилизаторе</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>~15 мА</t>
-        </is>
-      </c>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>СОПРОТИВЛЕНИЕ КАБЕЛЕЙ (одна жила, Ом)</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="n"/>
       <c r="C24" s="24" t="n"/>
       <c r="D24" s="24" t="n"/>
       <c r="E24" s="24" t="n"/>
       <c r="F24" s="24" t="n"/>
     </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Кабель</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>R@20°C</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>R@35°C</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>R@50°C</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>R@65°C</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>R петли@50°C</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>СОПРОТИВЛЕНИЕ КАБЕЛЕЙ (одна жила, Ом)</t>
-        </is>
-      </c>
-      <c r="B26" s="24" t="n"/>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Cable 9 (250м, 1.5мм²)</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>2.917</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>3.089</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>3.261</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>3.432</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>6.521</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Кабель</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>R@20°C</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>R@35°C</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>R@50°C</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>R@65°C</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>R петли@50°C</t>
-        </is>
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Cable 3 (15м, 1.5мм²)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>0.391</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Cable 9 (250м, 1.5мм²)</t>
+          <t>Cable 4 (15м, 1.5мм²)</t>
         </is>
       </c>
       <c r="B28" s="14" t="n">
-        <v>2.917</v>
+        <v>0.175</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>3.089</v>
+        <v>0.185</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>3.261</v>
+        <v>0.196</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>3.432</v>
+        <v>0.206</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>6.521</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>Cable 3 (15м, 1.5мм²)</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="C29" s="14" t="n">
-        <v>0.185</v>
-      </c>
-      <c r="D29" s="14" t="n">
-        <v>0.196</v>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>0.206</v>
-      </c>
-      <c r="F29" s="14" t="n">
         <v>0.391</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Cable 4 (15м, 1.5мм²)</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="C30" s="14" t="n">
-        <v>0.185</v>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>0.196</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>0.206</v>
-      </c>
-      <c r="F30" s="14" t="n">
-        <v>0.391</v>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="33" t="inlineStr">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>СВОДНАЯ ТАБЛИЦА: НАПРЯЖЕНИЕ НА КЛЕММАХ ТРАНСМИТТЕРА (В)</t>
         </is>
       </c>
-      <c r="B32" s="24" t="n"/>
-      <c r="C32" s="24" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="24" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Режим работы</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>I транс., мА</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>20°C</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>35°C</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>50°C</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>65°C</t>
         </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Минимальный (пуск, прогрев)</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="n">
+        <v>200</v>
+      </c>
+      <c r="C32" s="34" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D32" s="34" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="E32" s="34" t="n">
+        <v>21.31</v>
+      </c>
+      <c r="F32" s="34" t="n">
+        <v>21.17</v>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Номинальный (выходы ~12мА)</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="n">
+        <v>300</v>
+      </c>
+      <c r="C33" s="34" t="n">
+        <v>20.39</v>
+      </c>
+      <c r="D33" s="34" t="n">
+        <v>20.18</v>
+      </c>
+      <c r="E33" s="35" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="F33" s="35" t="n">
+        <v>19.76</v>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>Минимальный (холостой ход, выходы 4мА)</t>
+          <t>Паспортный (8 Вт / 24 В = 0.35 А)</t>
         </is>
       </c>
       <c r="B34" s="31" t="n">
-        <v>60</v>
-      </c>
-      <c r="C34" s="34" t="n">
-        <v>23.28</v>
-      </c>
-      <c r="D34" s="34" t="n">
-        <v>23.24</v>
-      </c>
-      <c r="E34" s="34" t="n">
-        <v>23.19</v>
-      </c>
-      <c r="F34" s="34" t="n">
-        <v>23.15</v>
+        <v>350</v>
+      </c>
+      <c r="C34" s="35" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="D34" s="35" t="n">
+        <v>19.55</v>
+      </c>
+      <c r="E34" s="35" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="F34" s="35" t="n">
+        <v>19.05</v>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Номинальный (выходы ~12мА)</t>
+          <t>Максимальный (с запасом 10%)</t>
         </is>
       </c>
       <c r="B35" s="31" t="n">
-        <v>120</v>
-      </c>
-      <c r="C35" s="34" t="n">
-        <v>22.56</v>
-      </c>
-      <c r="D35" s="34" t="n">
-        <v>22.47</v>
-      </c>
-      <c r="E35" s="34" t="n">
-        <v>22.39</v>
-      </c>
-      <c r="F35" s="34" t="n">
-        <v>22.3</v>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>Максимальный (выходы 20мА, полная нагрузка)</t>
-        </is>
-      </c>
-      <c r="B36" s="31" t="n">
-        <v>150</v>
-      </c>
-      <c r="C36" s="34" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="D36" s="34" t="n">
-        <v>22.09</v>
-      </c>
-      <c r="E36" s="34" t="n">
-        <v>21.98</v>
-      </c>
-      <c r="F36" s="34" t="n">
-        <v>21.88</v>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Аварийный (пусковой бросок)</t>
-        </is>
-      </c>
-      <c r="B37" s="31" t="n">
-        <v>200</v>
-      </c>
-      <c r="C37" s="34" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="D37" s="34" t="n">
-        <v>21.45</v>
-      </c>
-      <c r="E37" s="34" t="n">
-        <v>21.31</v>
-      </c>
-      <c r="F37" s="34" t="n">
-        <v>21.17</v>
+        <v>385</v>
+      </c>
+      <c r="C35" s="35" t="n">
+        <v>19.37</v>
+      </c>
+      <c r="D35" s="35" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="E35" s="35" t="n">
+        <v>18.83</v>
+      </c>
+      <c r="F35" s="35" t="n">
+        <v>18.56</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="36" t="inlineStr">
+        <is>
+          <t>Цветовая шкала:</t>
+        </is>
+      </c>
+      <c r="C36" s="37" t="inlineStr">
+        <is>
+          <t>&gt; 20 В</t>
+        </is>
+      </c>
+      <c r="D36" s="38" t="inlineStr">
+        <is>
+          <t>&lt; 20 В</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>&lt; 18 В</t>
+        </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="35" t="inlineStr">
-        <is>
-          <t>Цветовая шкала:</t>
-        </is>
-      </c>
-      <c r="C38" s="36" t="inlineStr">
-        <is>
-          <t>&gt; 20 В</t>
-        </is>
-      </c>
-      <c r="D38" s="37" t="inlineStr">
-        <is>
-          <t>&lt; 20 В</t>
-        </is>
-      </c>
-      <c r="E38" s="38" t="inlineStr">
-        <is>
-          <t>&lt; 18 В</t>
-        </is>
-      </c>
+      <c r="A38" s="40" t="inlineStr">
+        <is>
+          <t>ДЕТАЛЬНЫЙ РАСЧЁТ — ПАСПОРТНЫЙ РЕЖИМ (350 мА = 8 Вт, 65°C)</t>
+        </is>
+      </c>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>Ток одного трансмиттера</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t>350 мА</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="39" t="inlineStr">
-        <is>
-          <t>ДЕТАЛЬНЫЙ РАСЧЁТ — НАИХУДШИЙ СЛУЧАЙ (150 мА, 65°C)</t>
-        </is>
-      </c>
-      <c r="B40" s="24" t="n"/>
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>Суммарный ток в Cable 9 (оба трансмиттера)</t>
+        </is>
+      </c>
+      <c r="B40" s="42" t="inlineStr">
+        <is>
+          <t>700 мА</t>
+        </is>
+      </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="24" t="n"/>
       <c r="E40" s="24" t="n"/>
       <c r="F40" s="24" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="40" t="inlineStr">
-        <is>
-          <t>Ток одного трансмиттера</t>
-        </is>
-      </c>
-      <c r="B41" s="41" t="inlineStr">
-        <is>
-          <t>150 мА</t>
+      <c r="A41" s="41" t="inlineStr">
+        <is>
+          <t>R(Cable 9) при 65°C — одна жила</t>
+        </is>
+      </c>
+      <c r="B41" s="42" t="inlineStr">
+        <is>
+          <t>3.432 Ом</t>
         </is>
       </c>
       <c r="C41" s="24" t="n"/>
@@ -4020,14 +4019,14 @@
       <c r="F41" s="24" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="40" t="inlineStr">
-        <is>
-          <t>Суммарный ток в Cable 9 (оба трансмиттера)</t>
-        </is>
-      </c>
-      <c r="B42" s="41" t="inlineStr">
-        <is>
-          <t>300 мА</t>
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>R(Cable 9) при 65°C — петля (туда+обратно)</t>
+        </is>
+      </c>
+      <c r="B42" s="42" t="inlineStr">
+        <is>
+          <t>6.865 Ом</t>
         </is>
       </c>
       <c r="C42" s="24" t="n"/>
@@ -4036,14 +4035,14 @@
       <c r="F42" s="24" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="40" t="inlineStr">
-        <is>
-          <t>R(Cable 9) при 65°C — одна жила</t>
-        </is>
-      </c>
-      <c r="B43" s="41" t="inlineStr">
-        <is>
-          <t>3.432 Ом</t>
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>R(Cable 3/4) при 65°C — петля</t>
+        </is>
+      </c>
+      <c r="B43" s="42" t="inlineStr">
+        <is>
+          <t>0.412 Ом</t>
         </is>
       </c>
       <c r="C43" s="24" t="n"/>
@@ -4052,30 +4051,18 @@
       <c r="F43" s="24" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="40" t="inlineStr">
-        <is>
-          <t>R(Cable 9) при 65°C — петля (туда+обратно)</t>
-        </is>
-      </c>
-      <c r="B44" s="41" t="inlineStr">
-        <is>
-          <t>6.865 Ом</t>
-        </is>
-      </c>
-      <c r="C44" s="24" t="n"/>
-      <c r="D44" s="24" t="n"/>
-      <c r="E44" s="24" t="n"/>
-      <c r="F44" s="24" t="n"/>
+      <c r="A44" s="43" t="inlineStr"/>
+      <c r="B44" s="44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="40" t="inlineStr">
-        <is>
-          <t>R(Cable 3/4) при 65°C — петля</t>
-        </is>
-      </c>
-      <c r="B45" s="41" t="inlineStr">
-        <is>
-          <t>0.412 Ом</t>
+      <c r="A45" s="41" t="inlineStr">
+        <is>
+          <t>ΔU на Cable 9 (250 м)</t>
+        </is>
+      </c>
+      <c r="B45" s="42" t="inlineStr">
+        <is>
+          <t>4.81 В</t>
         </is>
       </c>
       <c r="C45" s="24" t="n"/>
@@ -4084,18 +4071,30 @@
       <c r="F45" s="24" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="42" t="inlineStr"/>
-      <c r="B46" s="43" t="inlineStr"/>
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>ΔU на Cable 3/4 (15 м)</t>
+        </is>
+      </c>
+      <c r="B46" s="42" t="inlineStr">
+        <is>
+          <t>0.14 В</t>
+        </is>
+      </c>
+      <c r="C46" s="24" t="n"/>
+      <c r="D46" s="24" t="n"/>
+      <c r="E46" s="24" t="n"/>
+      <c r="F46" s="24" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="40" t="inlineStr">
-        <is>
-          <t>ΔU на Cable 9 (250 м)</t>
-        </is>
-      </c>
-      <c r="B47" s="41" t="inlineStr">
-        <is>
-          <t>2.06 В</t>
+      <c r="A47" s="45" t="inlineStr">
+        <is>
+          <t>ИТОГО падение напряжения</t>
+        </is>
+      </c>
+      <c r="B47" s="46" t="inlineStr">
+        <is>
+          <t>4.95 В  (20.6%)</t>
         </is>
       </c>
       <c r="C47" s="24" t="n"/>
@@ -4104,30 +4103,18 @@
       <c r="F47" s="24" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="40" t="inlineStr">
-        <is>
-          <t>ΔU на Cable 3/4 (15 м)</t>
-        </is>
-      </c>
-      <c r="B48" s="41" t="inlineStr">
-        <is>
-          <t>0.06 В</t>
-        </is>
-      </c>
-      <c r="C48" s="24" t="n"/>
-      <c r="D48" s="24" t="n"/>
-      <c r="E48" s="24" t="n"/>
-      <c r="F48" s="24" t="n"/>
+      <c r="A48" s="43" t="inlineStr"/>
+      <c r="B48" s="44" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="44" t="inlineStr">
-        <is>
-          <t>ИТОГО падение напряжения</t>
-        </is>
-      </c>
-      <c r="B49" s="45" t="inlineStr">
-        <is>
-          <t>2.12 В  (8.8%)</t>
+      <c r="A49" s="41" t="inlineStr">
+        <is>
+          <t>V на Connection Box</t>
+        </is>
+      </c>
+      <c r="B49" s="42" t="inlineStr">
+        <is>
+          <t>19.19 В</t>
         </is>
       </c>
       <c r="C49" s="24" t="n"/>
@@ -4136,34 +4123,34 @@
       <c r="F49" s="24" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="42" t="inlineStr"/>
-      <c r="B50" s="43" t="inlineStr"/>
+      <c r="A50" s="45" t="inlineStr">
+        <is>
+          <t>V НА ТРАНСМИТТЕРЕ</t>
+        </is>
+      </c>
+      <c r="B50" s="46" t="inlineStr">
+        <is>
+          <t>19.05 В</t>
+        </is>
+      </c>
+      <c r="C50" s="24" t="n"/>
+      <c r="D50" s="24" t="n"/>
+      <c r="E50" s="24" t="n"/>
+      <c r="F50" s="24" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="40" t="inlineStr">
-        <is>
-          <t>V на Connection Box</t>
-        </is>
-      </c>
-      <c r="B51" s="41" t="inlineStr">
-        <is>
-          <t>21.94 В</t>
-        </is>
-      </c>
-      <c r="C51" s="24" t="n"/>
-      <c r="D51" s="24" t="n"/>
-      <c r="E51" s="24" t="n"/>
-      <c r="F51" s="24" t="n"/>
+      <c r="A51" s="43" t="inlineStr"/>
+      <c r="B51" s="44" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="44" t="inlineStr">
-        <is>
-          <t>V НА ТРАНСМИТТЕРЕ</t>
-        </is>
-      </c>
-      <c r="B52" s="45" t="inlineStr">
-        <is>
-          <t>21.88 В</t>
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>Мощность потерь в Cable 9</t>
+        </is>
+      </c>
+      <c r="B52" s="42" t="inlineStr">
+        <is>
+          <t>3.36 Вт</t>
         </is>
       </c>
       <c r="C52" s="24" t="n"/>
@@ -4172,18 +4159,30 @@
       <c r="F52" s="24" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="42" t="inlineStr"/>
-      <c r="B53" s="43" t="inlineStr"/>
+      <c r="A53" s="41" t="inlineStr">
+        <is>
+          <t>Мощность потерь в Cable 3/4</t>
+        </is>
+      </c>
+      <c r="B53" s="42" t="inlineStr">
+        <is>
+          <t>0.050 Вт</t>
+        </is>
+      </c>
+      <c r="C53" s="24" t="n"/>
+      <c r="D53" s="24" t="n"/>
+      <c r="E53" s="24" t="n"/>
+      <c r="F53" s="24" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="40" t="inlineStr">
-        <is>
-          <t>Мощность потерь в Cable 9</t>
-        </is>
-      </c>
-      <c r="B54" s="41" t="inlineStr">
-        <is>
-          <t>0.62 Вт</t>
+      <c r="A54" s="41" t="inlineStr">
+        <is>
+          <t>Суммарные тепловые потери</t>
+        </is>
+      </c>
+      <c r="B54" s="42" t="inlineStr">
+        <is>
+          <t>3.41 Вт</t>
         </is>
       </c>
       <c r="C54" s="24" t="n"/>
@@ -4191,95 +4190,109 @@
       <c r="E54" s="24" t="n"/>
       <c r="F54" s="24" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="40" t="inlineStr">
-        <is>
-          <t>Мощность потерь в Cable 3/4</t>
-        </is>
-      </c>
-      <c r="B55" s="41" t="inlineStr">
-        <is>
-          <t>0.009 Вт</t>
-        </is>
-      </c>
-      <c r="C55" s="24" t="n"/>
-      <c r="D55" s="24" t="n"/>
-      <c r="E55" s="24" t="n"/>
-      <c r="F55" s="24" t="n"/>
-    </row>
     <row r="56">
-      <c r="A56" s="40" t="inlineStr">
-        <is>
-          <t>Суммарные тепловые потери</t>
-        </is>
-      </c>
-      <c r="B56" s="41" t="inlineStr">
-        <is>
-          <t>0.63 Вт</t>
-        </is>
-      </c>
+      <c r="A56" s="47" t="inlineStr">
+        <is>
+          <t>РЕКОМЕНДАЦИИ / RECOMMENDATIONS</t>
+        </is>
+      </c>
+      <c r="B56" s="24" t="n"/>
       <c r="C56" s="24" t="n"/>
       <c r="D56" s="24" t="n"/>
       <c r="E56" s="24" t="n"/>
       <c r="F56" s="24" t="n"/>
     </row>
-    <row r="58">
-      <c r="A58" s="46" t="inlineStr">
-        <is>
-          <t>РЕКОМЕНДАЦИИ / RECOMMENDATIONS</t>
-        </is>
-      </c>
-      <c r="B58" s="24" t="n"/>
-      <c r="C58" s="24" t="n"/>
-      <c r="D58" s="24" t="n"/>
-      <c r="E58" s="24" t="n"/>
-      <c r="F58" s="24" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Рекомендация</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Параметр</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>V, В</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Падение, В</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Статус</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>1. Увеличить сечение Cable 9 до 2.5 мм²</t>
+        </is>
+      </c>
+      <c r="B58" s="32" t="inlineStr">
+        <is>
+          <t>V на трансмиттере (65°C, 350мА)</t>
+        </is>
+      </c>
+      <c r="C58" s="34" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="D58" s="14" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="E58" s="48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>2. Повысить напряжение источника до 27 В</t>
+        </is>
+      </c>
+      <c r="B59" s="32" t="inlineStr">
+        <is>
+          <t>V на трансмиттере (65°C, 350мА)</t>
+        </is>
+      </c>
+      <c r="C59" s="34" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="D59" s="14" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E59" s="48" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>1. Увеличить сечение Cable 9 до 2.5 мм²</t>
+          <t>3. Сократить Cable 9 до 100 м (перенести SCADA box)</t>
         </is>
       </c>
       <c r="B60" s="32" t="inlineStr">
         <is>
-          <t>V на трансмиттере (65°C, 150мА)</t>
+          <t>V на трансмиттере (65°C, 350мА)</t>
         </is>
       </c>
       <c r="C60" s="34" t="n">
-        <v>22.7</v>
+        <v>21.93</v>
       </c>
       <c r="D60" s="14" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="E60" s="47" t="inlineStr">
+        <v>2.07</v>
+      </c>
+      <c r="E60" s="48" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -4288,106 +4301,58 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>2. Повысить напряжение источника до 27 В</t>
+          <t>4. Отдельный БП 24VDC у Connection Box</t>
         </is>
       </c>
       <c r="B61" s="32" t="inlineStr">
         <is>
-          <t>V на трансмиттере (65°C, 150мА)</t>
+          <t>V на трансмиттере (без Cable 9)</t>
         </is>
       </c>
       <c r="C61" s="34" t="n">
-        <v>24.88</v>
+        <v>23.86</v>
       </c>
       <c r="D61" s="14" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="E61" s="47" t="inlineStr">
+        <v>0.14</v>
+      </c>
+      <c r="E61" s="48" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="16" t="inlineStr">
-        <is>
-          <t>3. Сократить Cable 9 до 100 м (перенести SCADA box)</t>
-        </is>
-      </c>
-      <c r="B62" s="32" t="inlineStr">
-        <is>
-          <t>V на трансмиттере (65°C, 150мА)</t>
-        </is>
-      </c>
-      <c r="C62" s="34" t="n">
-        <v>23.11</v>
-      </c>
-      <c r="D62" s="14" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="E62" s="47" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>4. Отдельный БП 24VDC у Connection Box</t>
-        </is>
-      </c>
-      <c r="B63" s="32" t="inlineStr">
-        <is>
-          <t>V на трансмиттере (без Cable 9)</t>
-        </is>
-      </c>
-      <c r="C63" s="34" t="n">
-        <v>23.94</v>
-      </c>
-      <c r="D63" s="14" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="E63" s="47" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="39">
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="B46:F46"/>
+    <mergeCell ref="A56:F56"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="B56:F56"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B39:F39"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="A32:F32"/>
     <mergeCell ref="B42:F42"/>
-    <mergeCell ref="B23:F23"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="B44:F44"/>
     <mergeCell ref="B53:F53"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="B40:F40"/>
     <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B55:F55"/>
-    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>